<commit_message>
Simplify dashboard export to Dashboard, Consolidado and Resumen
</commit_message>
<xml_diff>
--- a/reports/dashboard-template.xlsx
+++ b/reports/dashboard-template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R95a8ef986d9f4625"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="R006192f66c2f42e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gestiones" sheetId="3" r:id="Rd1f661f1576e44fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle" sheetId="4" r:id="R66c05b4d57f049c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd61b5aff2e2d4499"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="R3768e60c4b604412"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gestiones" sheetId="3" r:id="R05662dc67d2840ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle" sheetId="4" r:id="Ra56a7b99413447c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -245,13 +245,13 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -1183,7 +1183,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd203b46ae60547be"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R857997d58d1c460c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1213,7 +1213,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8ae2dde16c7c44f8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1f932a1e64814251"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1243,7 +1243,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a0ebea34e1348c5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7977089bc3ac47b9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1273,7 +1273,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc7dd7cd47b724bf1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f9c2bc7ec524d22"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1301,7 +1301,7 @@
     <x:tableColumn id="14" name="Entrega liquidadora"/>
     <x:tableColumn id="15" name="Nota débito"/>
     <x:tableColumn id="16" name="Ingreso GP"/>
-    <x:tableColumn id="17" name="Finalizado"/>
+    <x:tableColumn id="17" name="Finalizada"/>
     <x:tableColumn id="18" name="N1–N2 (h)"/>
     <x:tableColumn id="19" name="N2–N3 (h)"/>
     <x:tableColumn id="20" name="N3–N4 (h)"/>
@@ -1341,7 +1341,7 @@
     <x:tableColumn id="17" name="Entrega liquidadora"/>
     <x:tableColumn id="18" name="Nota débito"/>
     <x:tableColumn id="19" name="Ingreso GP"/>
-    <x:tableColumn id="20" name="Finalizado"/>
+    <x:tableColumn id="20" name="Finalizada"/>
     <x:tableColumn id="21" name="N1–N2 (h)"/>
     <x:tableColumn id="22" name="N2–N3 (h)"/>
     <x:tableColumn id="23" name="N3–N4 (h)"/>
@@ -1694,9 +1694,7 @@
       <x:c r="AH3" s="2"/>
     </x:row>
     <x:row r="4" ht="16" customHeight="1">
-      <x:c r="A4" s="9" t="str">
-        <x:v>Operación de bodega y logística de café</x:v>
-      </x:c>
+      <x:c r="A4" s="9" t="str"/>
       <x:c r="B4" s="9"/>
       <x:c r="C4" s="9"/>
       <x:c r="D4" s="9"/>
@@ -2701,30 +2699,30 @@
     </x:row>
     <x:row r="31" ht="12" customHeight="1">
       <x:c r="A31" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A31)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A31),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(1&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(1,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B31" s="71"/>
       <x:c r="C31" s="71"/>
       <x:c r="D31" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A31)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A31),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(1&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(1,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E31" s="71"/>
       <x:c r="F31" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A31)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A31),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(1&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(1,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G31" s="71"/>
       <x:c r="H31" s="71"/>
       <x:c r="I31" s="71"/>
       <x:c r="J31" s="71"/>
       <x:c r="K31" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A31)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A31),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(1&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(1,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L31" s="71"/>
       <x:c r="M31" s="71"/>
       <x:c r="N31" s="71"/>
       <x:c r="O31" s="71"/>
       <x:c r="P31" s="73" t="str">
-        <x:f>IF(ROWS($A$31:A31)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A31),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(1&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(1,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q31" s="73"/>
       <x:c r="R31" s="73"/>
@@ -2747,30 +2745,30 @@
     </x:row>
     <x:row r="32" ht="12" customHeight="1">
       <x:c r="A32" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A32)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A32),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(2&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(2,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B32" s="72"/>
       <x:c r="C32" s="72"/>
       <x:c r="D32" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A32)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A32),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(2&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(2,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E32" s="72"/>
       <x:c r="F32" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A32)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A32),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(2&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(2,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G32" s="72"/>
       <x:c r="H32" s="72"/>
       <x:c r="I32" s="72"/>
       <x:c r="J32" s="72"/>
       <x:c r="K32" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A32)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A32),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(2&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(2,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L32" s="72"/>
       <x:c r="M32" s="72"/>
       <x:c r="N32" s="72"/>
       <x:c r="O32" s="72"/>
       <x:c r="P32" s="74" t="str">
-        <x:f>IF(ROWS($A$31:A32)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A32),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(2&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(2,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q32" s="74"/>
       <x:c r="R32" s="74"/>
@@ -2793,30 +2791,30 @@
     </x:row>
     <x:row r="33" ht="12" customHeight="1">
       <x:c r="A33" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A33)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A33),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(3&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(3,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B33" s="71"/>
       <x:c r="C33" s="71"/>
       <x:c r="D33" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A33)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A33),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(3&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(3,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E33" s="71"/>
       <x:c r="F33" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A33)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A33),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(3&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(3,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G33" s="71"/>
       <x:c r="H33" s="71"/>
       <x:c r="I33" s="71"/>
       <x:c r="J33" s="71"/>
       <x:c r="K33" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A33)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A33),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(3&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(3,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L33" s="71"/>
       <x:c r="M33" s="71"/>
       <x:c r="N33" s="71"/>
       <x:c r="O33" s="71"/>
       <x:c r="P33" s="73" t="str">
-        <x:f>IF(ROWS($A$31:A33)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A33),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(3&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(3,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q33" s="73"/>
       <x:c r="R33" s="73"/>
@@ -2839,30 +2837,30 @@
     </x:row>
     <x:row r="34" ht="12" customHeight="1">
       <x:c r="A34" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A34)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A34),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(4&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(4,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B34" s="72"/>
       <x:c r="C34" s="72"/>
       <x:c r="D34" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A34)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A34),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(4&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(4,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E34" s="72"/>
       <x:c r="F34" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A34)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A34),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(4&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(4,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G34" s="72"/>
       <x:c r="H34" s="72"/>
       <x:c r="I34" s="72"/>
       <x:c r="J34" s="72"/>
       <x:c r="K34" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A34)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A34),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(4&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(4,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L34" s="72"/>
       <x:c r="M34" s="72"/>
       <x:c r="N34" s="72"/>
       <x:c r="O34" s="72"/>
       <x:c r="P34" s="74" t="str">
-        <x:f>IF(ROWS($A$31:A34)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A34),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(4&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(4,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q34" s="74"/>
       <x:c r="R34" s="74"/>
@@ -2885,30 +2883,30 @@
     </x:row>
     <x:row r="35" ht="12" customHeight="1">
       <x:c r="A35" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A35)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A35),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(5&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(5,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B35" s="71"/>
       <x:c r="C35" s="71"/>
       <x:c r="D35" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A35)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A35),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(5&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(5,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E35" s="71"/>
       <x:c r="F35" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A35)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A35),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(5&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(5,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G35" s="71"/>
       <x:c r="H35" s="71"/>
       <x:c r="I35" s="71"/>
       <x:c r="J35" s="71"/>
       <x:c r="K35" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A35)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A35),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(5&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(5,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L35" s="71"/>
       <x:c r="M35" s="71"/>
       <x:c r="N35" s="71"/>
       <x:c r="O35" s="71"/>
       <x:c r="P35" s="73" t="str">
-        <x:f>IF(ROWS($A$31:A35)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A35),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(5&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(5,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q35" s="73"/>
       <x:c r="R35" s="73"/>
@@ -2931,30 +2929,30 @@
     </x:row>
     <x:row r="36" ht="12" customHeight="1">
       <x:c r="A36" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A36)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A36),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(6&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(6,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B36" s="72"/>
       <x:c r="C36" s="72"/>
       <x:c r="D36" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A36)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A36),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(6&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(6,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E36" s="72"/>
       <x:c r="F36" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A36)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A36),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(6&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(6,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G36" s="72"/>
       <x:c r="H36" s="72"/>
       <x:c r="I36" s="72"/>
       <x:c r="J36" s="72"/>
       <x:c r="K36" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A36)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A36),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(6&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(6,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L36" s="72"/>
       <x:c r="M36" s="72"/>
       <x:c r="N36" s="72"/>
       <x:c r="O36" s="72"/>
       <x:c r="P36" s="74" t="str">
-        <x:f>IF(ROWS($A$31:A36)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A36),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(6&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(6,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q36" s="74"/>
       <x:c r="R36" s="74"/>
@@ -2977,30 +2975,30 @@
     </x:row>
     <x:row r="37" ht="12" customHeight="1">
       <x:c r="A37" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A37)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A37),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(7&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(7,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B37" s="71"/>
       <x:c r="C37" s="71"/>
       <x:c r="D37" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A37)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A37),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(7&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(7,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E37" s="71"/>
       <x:c r="F37" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A37)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A37),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(7&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(7,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G37" s="71"/>
       <x:c r="H37" s="71"/>
       <x:c r="I37" s="71"/>
       <x:c r="J37" s="71"/>
       <x:c r="K37" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A37)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A37),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(7&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(7,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L37" s="71"/>
       <x:c r="M37" s="71"/>
       <x:c r="N37" s="71"/>
       <x:c r="O37" s="71"/>
       <x:c r="P37" s="73" t="str">
-        <x:f>IF(ROWS($A$31:A37)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A37),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(7&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(7,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q37" s="73"/>
       <x:c r="R37" s="73"/>
@@ -3023,30 +3021,30 @@
     </x:row>
     <x:row r="38" ht="12" customHeight="1">
       <x:c r="A38" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A38)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A38),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(8&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(8,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B38" s="72"/>
       <x:c r="C38" s="72"/>
       <x:c r="D38" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A38)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A38),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(8&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(8,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E38" s="72"/>
       <x:c r="F38" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A38)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A38),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(8&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(8,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G38" s="72"/>
       <x:c r="H38" s="72"/>
       <x:c r="I38" s="72"/>
       <x:c r="J38" s="72"/>
       <x:c r="K38" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A38)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A38),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(8&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(8,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L38" s="72"/>
       <x:c r="M38" s="72"/>
       <x:c r="N38" s="72"/>
       <x:c r="O38" s="72"/>
       <x:c r="P38" s="74" t="str">
-        <x:f>IF(ROWS($A$31:A38)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A38),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(8&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(8,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q38" s="74"/>
       <x:c r="R38" s="74"/>
@@ -3069,30 +3067,30 @@
     </x:row>
     <x:row r="39" ht="12" customHeight="1">
       <x:c r="A39" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A39)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A39),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(9&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(9,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B39" s="71"/>
       <x:c r="C39" s="71"/>
       <x:c r="D39" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A39)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A39),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(9&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(9,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E39" s="71"/>
       <x:c r="F39" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A39)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A39),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(9&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(9,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G39" s="71"/>
       <x:c r="H39" s="71"/>
       <x:c r="I39" s="71"/>
       <x:c r="J39" s="71"/>
       <x:c r="K39" s="71" t="str">
-        <x:f>IF(ROWS($A$31:A39)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A39),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(9&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(9,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L39" s="71"/>
       <x:c r="M39" s="71"/>
       <x:c r="N39" s="71"/>
       <x:c r="O39" s="71"/>
       <x:c r="P39" s="73" t="str">
-        <x:f>IF(ROWS($A$31:A39)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A39),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(9&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(9,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q39" s="73"/>
       <x:c r="R39" s="73"/>
@@ -3115,30 +3113,30 @@
     </x:row>
     <x:row r="40" ht="12" customHeight="1">
       <x:c r="A40" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A40)&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(ROWS($A$31:A40),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(10&gt;Resumen!$B$4,"",INDEX(Gestiones!$A$6:$A$6,MATCH(10,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="B40" s="72"/>
       <x:c r="C40" s="72"/>
       <x:c r="D40" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A40)&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(ROWS($A$31:A40),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(10&gt;Resumen!$B$4,"",INDEX(Gestiones!$C$6:$C$6,MATCH(10,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="E40" s="72"/>
       <x:c r="F40" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A40)&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(ROWS($A$31:A40),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(10&gt;Resumen!$B$4,"",INDEX(Gestiones!$E$6:$E$6,MATCH(10,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="G40" s="72"/>
       <x:c r="H40" s="72"/>
       <x:c r="I40" s="72"/>
       <x:c r="J40" s="72"/>
       <x:c r="K40" s="72" t="str">
-        <x:f>IF(ROWS($A$31:A40)&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(ROWS($A$31:A40),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(10&gt;Resumen!$B$4,"",INDEX(Gestiones!$G$6:$G$6,MATCH(10,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="L40" s="72"/>
       <x:c r="M40" s="72"/>
       <x:c r="N40" s="72"/>
       <x:c r="O40" s="72"/>
       <x:c r="P40" s="74" t="str">
-        <x:f>IF(ROWS($A$31:A40)&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(ROWS($A$31:A40),Gestiones!$AC$6:$AC$6,0)))</x:f>
+        <x:f>IF(10&gt;Resumen!$B$4,"",INDEX(Gestiones!$U$6:$U$6,MATCH(10,Gestiones!$AC$6:$AC$6,0)))</x:f>
       </x:c>
       <x:c r="Q40" s="74"/>
       <x:c r="R40" s="74"/>
@@ -4032,7 +4030,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24e22b917474440d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra32d05739eb34aa5"/>
 </x:worksheet>
 </file>
 
@@ -4388,7 +4386,7 @@
         <x:v>Finalizadas</x:v>
       </x:c>
       <x:c r="B6" s="2" t="n">
-        <x:f>COUNTIFS(Gestiones!$H$6:$H$6,"Finalizado",Gestiones!$X$6:$X$6,1)</x:f>
+        <x:f>COUNTIFS(Gestiones!$H$6:$H$6,"Finalizada",Gestiones!$X$6:$X$6,1)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
@@ -4623,7 +4621,7 @@
         <x:v>En proceso</x:v>
       </x:c>
       <x:c r="B10" s="2" t="n">
-        <x:f>COUNTIFS(Gestiones!$X$6:$X$6,1,Gestiones!$H$6:$H$6,"&lt;&gt;Finalizado",Gestiones!$H$6:$H$6,"&lt;&gt;Anulado")</x:f>
+        <x:f>COUNTIFS(Gestiones!$X$6:$X$6,1,Gestiones!$H$6:$H$6,"&lt;&gt;Finalizada",Gestiones!$H$6:$H$6,"&lt;&gt;Anulada")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
@@ -7012,7 +7010,7 @@
         <x:v>Ingreso GP</x:v>
       </x:c>
       <x:c r="Q5" s="58" t="str">
-        <x:v>Finalizado</x:v>
+        <x:v>Finalizada</x:v>
       </x:c>
       <x:c r="R5" s="58" t="str">
         <x:v>N1–N2 (h)</x:v>
@@ -9044,7 +9042,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f45564725504a24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4cd22380b8f4a4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9294,7 +9292,7 @@
         <x:v>Ingreso GP</x:v>
       </x:c>
       <x:c r="T5" s="58" t="str">
-        <x:v>Finalizado</x:v>
+        <x:v>Finalizada</x:v>
       </x:c>
       <x:c r="U5" s="58" t="str">
         <x:v>N1–N2 (h)</x:v>
@@ -11319,7 +11317,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3183da4f62654b89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc55b18d01124f03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add daily state/warehouse Excel chart filters and data labels
</commit_message>
<xml_diff>
--- a/reports/dashboard-template.xlsx
+++ b/reports/dashboard-template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd61b5aff2e2d4499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="R3768e60c4b604412"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gestiones" sheetId="3" r:id="R05662dc67d2840ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle" sheetId="4" r:id="Ra56a7b99413447c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rcad8dd15810947b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="R585b9571c5b14fc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gestiones" sheetId="3" r:id="R358eb18d4d4648df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle" sheetId="4" r:id="Re51d0bced1ba4d49"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="205" formatCode="dd/mm/yyyy hh:mm"/>
     <x:numFmt numFmtId="206" formatCode="@"/>
   </x:numFmts>
-  <x:fonts count="17">
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -118,6 +118,17 @@
     <x:font>
       <x:sz val="9"/>
       <x:color rgb="FF34251F"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="8"/>
+      <x:color rgb="FF6B6B60"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF1D608B"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -232,7 +243,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="75">
+  <x:cellXfs count="86">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -454,6 +465,39 @@
     <x:xf numFmtId="201" fontId="16" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -478,7 +522,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Devoluciones por período</a:t>
+              <a:t>Devoluciones por Día</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -744,7 +788,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Motivos de devolución</a:t>
+              <a:t>Motivos de Devolución</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1163,7 +1207,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -1183,7 +1227,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R857997d58d1c460c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3d7e2714930849cc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1213,7 +1257,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1f932a1e64814251"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re23abeaa552c4c92"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1243,7 +1287,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7977089bc3ac47b9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcb8fd6541ecb449d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1273,7 +1317,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f9c2bc7ec524d22"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb6259f8810734450"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1930,19 +1974,25 @@
       <x:c r="AH9" s="2"/>
     </x:row>
     <x:row r="10" ht="12" customHeight="1">
-      <x:c r="A10" s="3"/>
-      <x:c r="B10" s="3"/>
-      <x:c r="C10" s="3"/>
-      <x:c r="D10" s="3"/>
+      <x:c r="A10" s="76" t="str">
+        <x:v>Mes</x:v>
+      </x:c>
+      <x:c r="B10" s="76"/>
+      <x:c r="C10" s="76"/>
+      <x:c r="D10" s="76"/>
       <x:c r="E10" s="3"/>
-      <x:c r="F10" s="3"/>
-      <x:c r="G10" s="3"/>
-      <x:c r="H10" s="3"/>
-      <x:c r="I10" s="3"/>
+      <x:c r="F10" s="76" t="str">
+        <x:v>Estado</x:v>
+      </x:c>
+      <x:c r="G10" s="76"/>
+      <x:c r="H10" s="76"/>
+      <x:c r="I10" s="76"/>
       <x:c r="J10" s="3"/>
-      <x:c r="K10" s="3"/>
-      <x:c r="L10" s="3"/>
-      <x:c r="M10" s="3"/>
+      <x:c r="K10" s="76" t="str">
+        <x:v>Bodega Destino</x:v>
+      </x:c>
+      <x:c r="L10" s="76"/>
+      <x:c r="M10" s="76"/>
       <x:c r="N10" s="3"/>
       <x:c r="O10" s="3"/>
       <x:c r="P10" s="3"/>
@@ -1966,19 +2016,25 @@
       <x:c r="AH10" s="2"/>
     </x:row>
     <x:row r="11" ht="12" customHeight="1">
-      <x:c r="A11" s="3"/>
-      <x:c r="B11" s="3"/>
-      <x:c r="C11" s="3"/>
-      <x:c r="D11" s="3"/>
+      <x:c r="A11" s="80" t="str">
+        <x:v>Todos los meses</x:v>
+      </x:c>
+      <x:c r="B11" s="81"/>
+      <x:c r="C11" s="81"/>
+      <x:c r="D11" s="82"/>
       <x:c r="E11" s="3"/>
-      <x:c r="F11" s="3"/>
-      <x:c r="G11" s="3"/>
-      <x:c r="H11" s="3"/>
-      <x:c r="I11" s="3"/>
+      <x:c r="F11" s="80" t="str">
+        <x:v>Todos</x:v>
+      </x:c>
+      <x:c r="G11" s="81"/>
+      <x:c r="H11" s="81"/>
+      <x:c r="I11" s="82"/>
       <x:c r="J11" s="3"/>
-      <x:c r="K11" s="3"/>
-      <x:c r="L11" s="3"/>
-      <x:c r="M11" s="3"/>
+      <x:c r="K11" s="80" t="str">
+        <x:v>Todas las bodegas</x:v>
+      </x:c>
+      <x:c r="L11" s="81"/>
+      <x:c r="M11" s="82"/>
       <x:c r="N11" s="3"/>
       <x:c r="O11" s="3"/>
       <x:c r="P11" s="3"/>
@@ -2002,19 +2058,19 @@
       <x:c r="AH11" s="2"/>
     </x:row>
     <x:row r="12" ht="12" customHeight="1">
-      <x:c r="A12" s="3"/>
-      <x:c r="B12" s="3"/>
-      <x:c r="C12" s="3"/>
-      <x:c r="D12" s="3"/>
+      <x:c r="A12" s="83"/>
+      <x:c r="B12" s="84"/>
+      <x:c r="C12" s="84"/>
+      <x:c r="D12" s="85"/>
       <x:c r="E12" s="3"/>
-      <x:c r="F12" s="3"/>
-      <x:c r="G12" s="3"/>
-      <x:c r="H12" s="3"/>
-      <x:c r="I12" s="3"/>
+      <x:c r="F12" s="83"/>
+      <x:c r="G12" s="84"/>
+      <x:c r="H12" s="84"/>
+      <x:c r="I12" s="85"/>
       <x:c r="J12" s="3"/>
-      <x:c r="K12" s="3"/>
-      <x:c r="L12" s="3"/>
-      <x:c r="M12" s="3"/>
+      <x:c r="K12" s="83"/>
+      <x:c r="L12" s="84"/>
+      <x:c r="M12" s="85"/>
       <x:c r="N12" s="3"/>
       <x:c r="O12" s="3"/>
       <x:c r="P12" s="3"/>
@@ -3706,9 +3762,7 @@
       <x:c r="AH54" s="2"/>
     </x:row>
     <x:row r="55" ht="12" customHeight="1">
-      <x:c r="A55" s="46" t="str">
-        <x:v>Los filtros de Excel acotan la selección exportada desde la web.</x:v>
-      </x:c>
+      <x:c r="A55" s="46" t="str"/>
       <x:c r="B55" s="46"/>
       <x:c r="C55" s="46"/>
       <x:c r="D55" s="46"/>
@@ -3744,9 +3798,7 @@
       <x:c r="AH55" s="2"/>
     </x:row>
     <x:row r="56" ht="12" customHeight="1">
-      <x:c r="A56" s="46" t="str">
-        <x:v>Motivos y gestores: siete categorías principales del reporte y otras.</x:v>
-      </x:c>
+      <x:c r="A56" s="46" t="str"/>
       <x:c r="B56" s="46"/>
       <x:c r="C56" s="46"/>
       <x:c r="D56" s="46"/>
@@ -4017,8 +4069,14 @@
     <x:mergeCell ref="P38:R38"/>
     <x:mergeCell ref="P39:R39"/>
     <x:mergeCell ref="P40:R40"/>
+    <x:mergeCell ref="A10:D10"/>
+    <x:mergeCell ref="A11:D12"/>
+    <x:mergeCell ref="F10:I10"/>
+    <x:mergeCell ref="F11:I12"/>
+    <x:mergeCell ref="K10:M10"/>
+    <x:mergeCell ref="K11:M12"/>
   </x:mergeCells>
-  <x:dataValidations count="3">
+  <x:dataValidations count="8">
     <x:dataValidation type="list" sqref="A52">
       <x:formula1>INDIRECT("Resumen!$AA$2:$AA$2")</x:formula1>
     </x:dataValidation>
@@ -4028,9 +4086,26 @@
     <x:dataValidation type="list" sqref="L52">
       <x:formula1>INDIRECT("Resumen!$AC$2:$AC$2")</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="A11">
+      <x:formula1>INDIRECT("Resumen!$BP$2:$BP$2")</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F11">
+      <x:formula1>INDIRECT("Resumen!$AC$2:$AC$2")</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K11">
+      <x:formula1>INDIRECT("Resumen!$BQ$2:$BQ$2")</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="date" operator="between" sqref="R52">
+      <x:formula1>1</x:formula1>
+      <x:formula2>2958465</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="date" operator="between" sqref="V52">
+      <x:formula1>1</x:formula1>
+      <x:formula2>2958465</x:formula2>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra32d05739eb34aa5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95f570e48cad4215"/>
 </x:worksheet>
 </file>
 
@@ -9042,7 +9117,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4cd22380b8f4a4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cb63a958d61473e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11317,7 +11392,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc55b18d01124f03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8d980ba0401461c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>